<commit_message>
fix v4.5.7: 样本量变化表 — average team member response rate公式更正 0.785 -> 0.914
Customer correction: response rate calculation was wrong.

Old (wrong): Final_dyads / T1_submitted ≈ 0.785
  This treats T1_submitted (after attention/dup screening) as the
  baseline, which doubly penalizes (initial drop + cleaning drop).

New (per customer guidance):
  - average team member response rate among retained teams
    = avg_followers_per_leader / 5 (initial invites per team)
    = 4.57 / 5 = 0.914
  - overall follower retention rate (sample-level, not in table currently
    but derivable from R49/450)
    = Final_dyads / 450
    = 361 / 450 = 0.802

R54 (team member response rate_j, per-team) and R55 (average team member
response rate) both now show 0.914.

Initial invite N=450 = 90 leaders × 5 invites/team is given by spec
(R2 of the table is already pre-filled with 450).

189/189 + 10/10 PASS.
</commit_message>
<xml_diff>
--- a/results/样本量变化表.xlsx
+++ b/results/样本量变化表.xlsx
@@ -2242,7 +2242,7 @@
         </is>
       </c>
       <c r="C54" s="14" t="n">
-        <v>0.785</v>
+        <v>0.914</v>
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
@@ -2262,7 +2262,7 @@
         </is>
       </c>
       <c r="C55" s="14" t="n">
-        <v>0.785</v>
+        <v>0.914</v>
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
sync v4.5.7: 样本量变化表 response rate 0.785 -> 0.914 (avg/5)
</commit_message>
<xml_diff>
--- a/results/样本量变化表.xlsx
+++ b/results/样本量变化表.xlsx
@@ -2242,7 +2242,7 @@
         </is>
       </c>
       <c r="C54" s="14" t="n">
-        <v>0.785</v>
+        <v>0.914</v>
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
@@ -2262,7 +2262,7 @@
         </is>
       </c>
       <c r="C55" s="14" t="n">
-        <v>0.785</v>
+        <v>0.914</v>
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>

</xml_diff>